<commit_message>
Auto-registro SGC: Folio SALIDA-REM-OUT-2026-0001
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,6 +465,54 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REM-OUT-2026-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A17</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" t="n">
+        <v>495.9777777777778</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PRIME-003-OC2602-0711-T4-CAL14</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Marvin Flores</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Se regresa el atado a almacen..!!!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio SALIDA-REM-OUT-2026-0002
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,54 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>Se regresa el atado a almacen..!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REM-OUT-2026-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A01</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>225.4444444444444</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>OT-0001</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Bryan</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>ksjdlksaj</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio SALIDA-REM-OUT-2026-0003
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,6 +561,54 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>ksjdlksaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REM-OUT-2026-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A17</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="n">
+        <v>450.8888888888889</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>OT-0001-AJHDKSAJH</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>jsadsa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio RECHAZO-REJ-OUT-2026-0004
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,26 @@
           <t>Observaciones</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Hojas_Defectuosas</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Tipo_Defecto</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Gravedad_Defecto</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Accion_Defecto</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -515,6 +535,10 @@
           <t>Se regresa el atado a almacen..!!!</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -563,6 +587,10 @@
           <t>ksjdlksaj</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -609,6 +637,72 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>jsadsa</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REJ-OUT-2026-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>18:38</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A01</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>45.08888888888889</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Rechazo de Láminas - Defecto en Proceso</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Operador Láser</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Raya / Rasguño</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Leve</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Scrap / Desecho</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio SALIDA-REM-OUT-2026-0005
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -706,6 +706,56 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REM-OUT-2026-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A03</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>360.7111111111111</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>INT 035</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Marvin Flores</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio RECHAZO-REJ-OUT-2026-0006
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,6 +756,68 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REJ-OUT-2026-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A17</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>45.08888888888889</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Rechazo de Láminas - Defecto en Proceso</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Operador Láser</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Raya / Rasguño</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Leve</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Scrap / Desecho</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio SALIDA-REM-OUT-2026-0007
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,6 +818,56 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REM-OUT-2026-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>18:58</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A01</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>405.8</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>INT-0026</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Marvin Flores</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio RECHAZO-REJ-OUT-2026-0002
</commit_message>
<xml_diff>
--- a/BD_Salidas_Incoming.xlsx
+++ b/BD_Salidas_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,11 +520,7 @@
       <c r="G2" t="n">
         <v>360.7111111111111</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Juan P</t>
@@ -541,6 +537,68 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REJ-OUT-2026-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>18/06/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>INC-2026-0001-A03</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>45.08888888888889</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Rechazo de Láminas - Defecto en Proceso</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>zcxzc</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Raya / Rasguño</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Reclamación a Proveedor</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>